<commit_message>
Met à jour carnet-terrain.xlsx (suivi personnel des visites)
</commit_message>
<xml_diff>
--- a/carnet-terrain.xlsx
+++ b/carnet-terrain.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\EXPAT\MAURICE APP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{145F27BA-1B05-488D-9963-E05AEB4607C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{085BFBBA-2F7D-4AD1-8C00-D41E1A72863F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="140">
   <si>
     <t>Date visite</t>
   </si>
@@ -438,6 +438,9 @@
   </si>
   <si>
     <t xml:space="preserve">Superbe parc. Organisation rodée voire un peu mécanique pour orienter vers les différentes activités payantes. Gratuit: balade de tout le site avec ponts, cascades, points devue et 23 couelurs. Parc aux tortues géantes, espace jeux enfants. Activités pyantes: tyroliennes, luge, quad,.. </t>
+  </si>
+  <si>
+    <t>Théo aux fourneaux</t>
   </si>
 </sst>
 </file>
@@ -589,9 +592,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -609,6 +609,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1047,26 +1050,26 @@
       <c r="E4" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="16" t="s">
         <v>98</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="I4" s="20" t="s">
+      <c r="I4" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="J4" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="K4" s="20" t="s">
+      <c r="K4" s="17" t="s">
         <v>102</v>
       </c>
       <c r="L4" s="12"/>
-      <c r="M4" s="21" t="s">
+      <c r="M4" s="18" t="s">
         <v>103</v>
       </c>
       <c r="N4" s="11"/>
@@ -1075,7 +1078,7 @@
       <c r="A5" s="10">
         <v>46214</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="19" t="s">
         <v>104</v>
       </c>
       <c r="C5" s="7" t="s">
@@ -1085,24 +1088,24 @@
       <c r="E5" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="21">
         <v>2304800735</v>
       </c>
       <c r="H5" s="7"/>
-      <c r="I5" s="22" t="s">
+      <c r="I5" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="J5" s="22" t="s">
+      <c r="J5" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="K5" s="22" t="s">
+      <c r="K5" s="19" t="s">
         <v>108</v>
       </c>
       <c r="L5" s="8"/>
-      <c r="M5" s="25" t="s">
+      <c r="M5" s="22" t="s">
         <v>109</v>
       </c>
       <c r="N5" s="7"/>
@@ -1111,27 +1114,27 @@
       <c r="A6" s="10">
         <v>46199</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="17" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="17" t="s">
         <v>110</v>
       </c>
       <c r="D6" s="11"/>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="17" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
-      <c r="I6" s="20" t="s">
+      <c r="I6" s="17" t="s">
         <v>111</v>
       </c>
       <c r="J6" s="11"/>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="17" t="s">
         <v>113</v>
       </c>
       <c r="L6" s="12"/>
-      <c r="M6" s="21" t="s">
+      <c r="M6" s="18" t="s">
         <v>114</v>
       </c>
       <c r="N6" s="11"/>
@@ -1140,28 +1143,28 @@
       <c r="A7" s="10">
         <v>46206</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="11"/>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="17" t="s">
         <v>115</v>
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
-      <c r="I7" s="20" t="s">
+      <c r="I7" s="17" t="s">
         <v>122</v>
       </c>
       <c r="J7" s="11"/>
-      <c r="K7" s="20" t="s">
+      <c r="K7" s="17" t="s">
         <v>117</v>
       </c>
       <c r="L7" s="12"/>
-      <c r="M7" s="21" t="s">
+      <c r="M7" s="18" t="s">
         <v>118</v>
       </c>
       <c r="N7" s="11"/>
@@ -1170,34 +1173,34 @@
       <c r="A8" s="6">
         <v>46209</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="19" t="s">
         <v>120</v>
       </c>
       <c r="D8" s="7"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="21">
         <v>23057198529</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="19" t="s">
         <v>125</v>
       </c>
       <c r="J8" s="7"/>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="19" t="s">
         <v>124</v>
       </c>
       <c r="L8" s="8"/>
-      <c r="M8" s="25" t="s">
+      <c r="M8" s="22" t="s">
         <v>123</v>
       </c>
       <c r="N8" s="7"/>
@@ -1213,27 +1216,27 @@
         <v>16</v>
       </c>
       <c r="D9" s="11"/>
-      <c r="E9" s="20" t="s">
+      <c r="E9" s="17" t="s">
         <v>134</v>
       </c>
       <c r="F9" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="16" t="s">
         <v>132</v>
       </c>
       <c r="H9" s="11"/>
-      <c r="I9" s="20" t="s">
+      <c r="I9" s="17" t="s">
         <v>135</v>
       </c>
-      <c r="J9" s="20" t="s">
+      <c r="J9" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="K9" s="20" t="s">
+      <c r="K9" s="17" t="s">
         <v>129</v>
       </c>
       <c r="L9" s="12"/>
-      <c r="M9" s="21" t="s">
+      <c r="M9" s="18" t="s">
         <v>130</v>
       </c>
       <c r="N9" s="11"/>
@@ -1242,7 +1245,7 @@
       <c r="A10" s="6">
         <v>46215</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="19" t="s">
         <v>136</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -1255,21 +1258,27 @@
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="22" t="s">
+      <c r="I10" s="19" t="s">
         <v>137</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="8"/>
-      <c r="M10" s="25" t="s">
+      <c r="M10" s="22" t="s">
         <v>138</v>
       </c>
       <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
+      <c r="A11" s="10">
+        <v>46217</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>16</v>
+      </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
@@ -4354,10 +4363,10 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="17"/>
+      <c r="B4" s="24"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
@@ -4464,10 +4473,10 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="17"/>
+      <c r="B19" s="24"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
@@ -4582,10 +4591,10 @@
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="B35" s="17"/>
+      <c r="B35" s="24"/>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
@@ -4612,10 +4621,10 @@
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
+      <c r="A40" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="B40" s="17"/>
+      <c r="B40" s="24"/>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="15" t="s">
@@ -4633,28 +4642,28 @@
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="B45" s="17"/>
+      <c r="B45" s="24"/>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="18" t="s">
+      <c r="A46" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B46" s="17"/>
+      <c r="B46" s="24"/>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
+      <c r="A48" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="17"/>
+      <c r="B48" s="24"/>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B49" s="17"/>
+      <c r="B49" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>